<commit_message>
Auto pipeline update 2026-01-23 16:11:38
</commit_message>
<xml_diff>
--- a/Productivity Summaries/Gang Productivity Buckets.xlsx
+++ b/Productivity Summaries/Gang Productivity Buckets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Productivity Summaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57DA8DBD-D332-4B9F-A6E6-2752A451199A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D72420E-B936-4A8B-A0A3-9C751683CCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{BD6F8336-0C2F-460A-A555-A39B18127C6E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8477" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8488" uniqueCount="586">
   <si>
     <t>Ajay Kumar</t>
   </si>
@@ -1789,13 +1789,22 @@
   </si>
   <si>
     <t>Zakir Hussain</t>
+  </si>
+  <si>
+    <t>&gt;=200</t>
+  </si>
+  <si>
+    <t>Gang-Months Share</t>
+  </si>
+  <si>
+    <t>MT (Output) Share</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1808,6 +1817,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1842,10 +1858,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1853,9 +1870,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1868,6 +1887,1235 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Monthly Gang Buckets'!$J$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Gang-Months Share</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="50000"/>
+                <a:lumOff val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Monthly Gang Buckets'!$G$5:$G$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>&lt;80</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>80-100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100-120</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>120-140</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>140-160</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>160-180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>180-200</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>&gt;=200</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Monthly Gang Buckets'!$J$5:$J$12</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.6194861851672322</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.592341250605914E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.398448860882211E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.622879301987397E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.65341735336888E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.6354823073194376E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.7629665535627727E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.3858458555501697E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-343C-4854-9F25-1E46EF0F62A1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Monthly Gang Buckets'!$K$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>MT (Output) Share</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="002060"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Monthly Gang Buckets'!$G$5:$G$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>&lt;80</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>80-100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100-120</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>120-140</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>140-160</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>160-180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>180-200</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>&gt;=200</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Monthly Gang Buckets'!$K$5:$K$12</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.2313005660985599</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.567668376889225E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.2826013574873092E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.2619138958610014E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.9420397951074301E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.0589465455989245E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6.4253521836251742E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.27331421235574938</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-343C-4854-9F25-1E46EF0F62A1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="31"/>
+        <c:overlap val="1"/>
+        <c:axId val="353890447"/>
+        <c:axId val="353881327"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$H$4</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$G$5:$G$12</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="8"/>
+                      <c:pt idx="0">
+                        <c:v>&lt;80</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>80-100</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>100-120</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>120-140</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>140-160</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>160-180</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>180-200</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>&gt;=200</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$H$5:$H$12</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="8"/>
+                      <c:pt idx="0">
+                        <c:v>1278</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>136</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>132</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>116</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>96</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>75</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>57</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>173</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-343C-4854-9F25-1E46EF0F62A1}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+            <c15:filteredBarSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$I$4</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="1"/>
+                    </c:strCache>
+                  </c:strRef>
+                </c:tx>
+                <c:spPr>
+                  <a:solidFill>
+                    <a:schemeClr val="accent2"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:invertIfNegative val="0"/>
+                <c:cat>
+                  <c:strRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$G$5:$G$12</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:strCache>
+                      <c:ptCount val="8"/>
+                      <c:pt idx="0">
+                        <c:v>&lt;80</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>80-100</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>100-120</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>120-140</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>140-160</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>160-180</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>180-200</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>&gt;=200</c:v>
+                      </c:pt>
+                    </c:strCache>
+                  </c:strRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>'Monthly Gang Buckets'!$I$5:$I$12</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="8"/>
+                      <c:pt idx="0">
+                        <c:v>36549.75</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>11958.31</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>14668.22</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>14635.53</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>14130.07</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>12734.62</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>10153.24</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>43188.68</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-343C-4854-9F25-1E46EF0F62A1}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredBarSeries>
+          </c:ext>
+        </c:extLst>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="353890447"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="353881327"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="353881327"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="90000"/>
+                  <a:alpha val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="353890447"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>511175</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>161924</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F08093B3-B155-4954-8988-B61024B8A0E6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10915,7 +12163,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F48BD1-4C83-4BAC-B843-586717BD5AFD}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G2081"/>
+  <dimension ref="A1:K2081"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.1796875" customWidth="1"/>
@@ -10925,17 +12173,17 @@
     <col min="6" max="6" width="15.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>129</v>
       </c>
@@ -10945,8 +12193,17 @@
       <c r="C4" s="2" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="G4" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>337</v>
       </c>
@@ -10956,8 +12213,35 @@
       <c r="C5">
         <v>36549.75</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="3">
+        <f>B5/SUM($B$5:$B$15)</f>
+        <v>0.6194861851672322</v>
+      </c>
+      <c r="E5" s="3">
+        <f>C5/SUM($C$5:$C$15)</f>
+        <v>0.2313005660985599</v>
+      </c>
+      <c r="G5" t="s">
+        <v>337</v>
+      </c>
+      <c r="H5">
+        <f>B5</f>
+        <v>1278</v>
+      </c>
+      <c r="I5">
+        <f>C5</f>
+        <v>36549.75</v>
+      </c>
+      <c r="J5" s="3">
+        <f>H5/SUM($H$5:$H$12)</f>
+        <v>0.6194861851672322</v>
+      </c>
+      <c r="K5" s="3">
+        <f>I5/SUM($I$5:$I$12)</f>
+        <v>0.2313005660985599</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>338</v>
       </c>
@@ -10967,8 +12251,35 @@
       <c r="C6">
         <v>11958.31</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <f t="shared" ref="D6:D15" si="0">B6/SUM($B$5:$B$15)</f>
+        <v>6.592341250605914E-2</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" ref="E6:E15" si="1">C6/SUM($C$5:$C$15)</f>
+        <v>7.567668376889225E-2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>338</v>
+      </c>
+      <c r="H6">
+        <f t="shared" ref="H6:H11" si="2">B6</f>
+        <v>136</v>
+      </c>
+      <c r="I6">
+        <f t="shared" ref="I6:I11" si="3">C6</f>
+        <v>11958.31</v>
+      </c>
+      <c r="J6" s="3">
+        <f t="shared" ref="J6:J12" si="4">H6/SUM($H$5:$H$12)</f>
+        <v>6.592341250605914E-2</v>
+      </c>
+      <c r="K6" s="3">
+        <f t="shared" ref="K6:K12" si="5">I6/SUM($I$5:$I$12)</f>
+        <v>7.567668376889225E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>339</v>
       </c>
@@ -10978,8 +12289,35 @@
       <c r="C7">
         <v>14668.22</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>6.398448860882211E-2</v>
+      </c>
+      <c r="E7" s="3">
+        <f t="shared" si="1"/>
+        <v>9.2826013574873092E-2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>339</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>132</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>14668.22</v>
+      </c>
+      <c r="J7" s="3">
+        <f t="shared" si="4"/>
+        <v>6.398448860882211E-2</v>
+      </c>
+      <c r="K7" s="3">
+        <f t="shared" si="5"/>
+        <v>9.2826013574873092E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>340</v>
       </c>
@@ -10989,8 +12327,35 @@
       <c r="C8">
         <v>14635.53</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>5.622879301987397E-2</v>
+      </c>
+      <c r="E8" s="3">
+        <f t="shared" si="1"/>
+        <v>9.2619138958610014E-2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>340</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="2"/>
+        <v>116</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>14635.53</v>
+      </c>
+      <c r="J8" s="3">
+        <f t="shared" si="4"/>
+        <v>5.622879301987397E-2</v>
+      </c>
+      <c r="K8" s="3">
+        <f t="shared" si="5"/>
+        <v>9.2619138958610014E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>341</v>
       </c>
@@ -11000,8 +12365,35 @@
       <c r="C9">
         <v>14130.07</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>4.65341735336888E-2</v>
+      </c>
+      <c r="E9" s="3">
+        <f t="shared" si="1"/>
+        <v>8.9420397951074301E-2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>341</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="2"/>
+        <v>96</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>14130.07</v>
+      </c>
+      <c r="J9" s="3">
+        <f t="shared" si="4"/>
+        <v>4.65341735336888E-2</v>
+      </c>
+      <c r="K9" s="3">
+        <f t="shared" si="5"/>
+        <v>8.9420397951074301E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>342</v>
       </c>
@@ -11011,8 +12403,35 @@
       <c r="C10">
         <v>12734.62</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
+        <f t="shared" si="0"/>
+        <v>3.6354823073194376E-2</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" si="1"/>
+        <v>8.0589465455989245E-2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>342</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>12734.62</v>
+      </c>
+      <c r="J10" s="3">
+        <f t="shared" si="4"/>
+        <v>3.6354823073194376E-2</v>
+      </c>
+      <c r="K10" s="3">
+        <f t="shared" si="5"/>
+        <v>8.0589465455989245E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>343</v>
       </c>
@@ -11022,8 +12441,35 @@
       <c r="C11">
         <v>10153.24</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="3">
+        <f t="shared" si="0"/>
+        <v>2.7629665535627727E-2</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="1"/>
+        <v>6.4253521836251742E-2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>343</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>57</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>10153.24</v>
+      </c>
+      <c r="J11" s="3">
+        <f t="shared" si="4"/>
+        <v>2.7629665535627727E-2</v>
+      </c>
+      <c r="K11" s="3">
+        <f t="shared" si="5"/>
+        <v>6.4253521836251742E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>344</v>
       </c>
@@ -11033,8 +12479,35 @@
       <c r="C12">
         <v>11491.96</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12" s="3">
+        <f t="shared" si="0"/>
+        <v>2.6175472612699952E-2</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" si="1"/>
+        <v>7.2725445552486848E-2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>583</v>
+      </c>
+      <c r="H12">
+        <f>SUM(B12:B15)</f>
+        <v>173</v>
+      </c>
+      <c r="I12">
+        <f>SUM(C12:C15)</f>
+        <v>43188.68</v>
+      </c>
+      <c r="J12" s="3">
+        <f t="shared" si="4"/>
+        <v>8.3858458555501697E-2</v>
+      </c>
+      <c r="K12" s="3">
+        <f t="shared" si="5"/>
+        <v>0.27331421235574938</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>345</v>
       </c>
@@ -11044,8 +12517,16 @@
       <c r="C13">
         <v>9393.1</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" s="3">
+        <f t="shared" si="0"/>
+        <v>1.9389238972370333E-2</v>
+      </c>
+      <c r="E13" s="3">
+        <f t="shared" si="1"/>
+        <v>5.9443069991460484E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>346</v>
       </c>
@@ -11055,8 +12536,16 @@
       <c r="C14">
         <v>8929.44</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14" s="3">
+        <f t="shared" si="0"/>
+        <v>1.6965584100824042E-2</v>
+      </c>
+      <c r="E14" s="3">
+        <f t="shared" si="1"/>
+        <v>5.6508855106891964E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>347</v>
       </c>
@@ -11065,6 +12554,14 @@
       </c>
       <c r="C15">
         <v>13374.18</v>
+      </c>
+      <c r="D15" s="3">
+        <f t="shared" si="0"/>
+        <v>2.1328162869607366E-2</v>
+      </c>
+      <c r="E15" s="3">
+        <f t="shared" si="1"/>
+        <v>8.4636841704910093E-2</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -56703,5 +58200,6 @@
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>